<commit_message>
change phieuXuatHang font size to 9
</commit_message>
<xml_diff>
--- a/public/pxh.xlsx
+++ b/public/pxh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diepm\Desktop\git\diepgia-management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDEC1FF-81F2-446F-B8A0-60553674952F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49910A7F-7039-4452-B43E-8C73D9F6C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -105,34 +105,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -142,12 +124,13 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -162,7 +145,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -171,54 +154,39 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -230,51 +198,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -560,100 +523,101 @@
   <sheetFormatPr defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="4.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="7" width="9.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="9.2109375" customWidth="1"/>
+    <col min="6" max="6" width="7.35546875" customWidth="1"/>
+    <col min="7" max="7" width="8.640625" customWidth="1"/>
+    <col min="8" max="8" width="14.0703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
       <c r="G1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="17"/>
+      <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="17.25" x14ac:dyDescent="0.45">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8" t="s">
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" ht="17.649999999999999" x14ac:dyDescent="0.5">
-      <c r="A5" s="2" t="s">
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="1:8" ht="13.9" x14ac:dyDescent="0.4">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="1:8" ht="17.649999999999999" x14ac:dyDescent="0.5">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:8" ht="13.9" x14ac:dyDescent="0.4">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="9"/>
+      <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:8" ht="13.9" x14ac:dyDescent="0.4">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="7"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="8"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -661,46 +625,46 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="16"/>
+      <c r="H9" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -712,5 +676,6 @@
     <mergeCell ref="H8:H9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="11" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change state loading sanpham
</commit_message>
<xml_diff>
--- a/public/pxh.xlsx
+++ b/public/pxh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diepm\Desktop\git\diepgia-management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFACAC8-8D7D-47A6-8F49-911EA79EE0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2680CEE-F773-4522-ADB2-E887F8AE3430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -226,18 +226,18 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -523,8 +523,8 @@
   <sheetFormatPr defaultRowHeight="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" customWidth="1"/>
     <col min="6" max="6" width="8.92578125" customWidth="1"/>
@@ -540,11 +540,11 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
@@ -554,23 +554,23 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" ht="17.25" x14ac:dyDescent="0.45">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
     </row>
     <row r="4" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
@@ -585,8 +585,8 @@
       <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="13.9" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
@@ -625,16 +625,16 @@
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="7" t="s">
@@ -646,15 +646,15 @@
       <c r="G8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="15" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
       <c r="E9" s="8" t="s">
         <v>16</v>
       </c>
@@ -664,7 +664,7 @@
       <c r="G9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="13"/>
+      <c r="H9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>